<commit_message>
Merged PR 2549: Merge planningmodulenewscenarios to master
</commit_message>
<xml_diff>
--- a/src/main/resources/Organizational_DeskReview_Field_Values.xlsx
+++ b/src/main/resources/Organizational_DeskReview_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B164733-7515-4E55-A531-43CC3255CA75}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C549426-EBDA-47CA-BD97-FB7828A38ECB}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="6" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
updated new test cases in Site Visits
</commit_message>
<xml_diff>
--- a/src/main/resources/Organizational_DeskReview_Field_Values.xlsx
+++ b/src/main/resources/Organizational_DeskReview_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21727"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C549426-EBDA-47CA-BD97-FB7828A38ECB}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53DA0360-8FF9-43CA-9C55-A0A6EE758A3D}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="6" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="5" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -18,9 +18,10 @@
     <sheet name="Award" sheetId="9" r:id="rId3"/>
     <sheet name="Sheet1" sheetId="4" r:id="rId4"/>
     <sheet name="Edition" sheetId="3" r:id="rId5"/>
-    <sheet name="Program" sheetId="6" r:id="rId6"/>
-    <sheet name="Fiscal" sheetId="7" r:id="rId7"/>
-    <sheet name="Form Fields" sheetId="5" r:id="rId8"/>
+    <sheet name="Edition1" sheetId="10" r:id="rId6"/>
+    <sheet name="Program" sheetId="6" r:id="rId7"/>
+    <sheet name="Fiscal" sheetId="7" r:id="rId8"/>
+    <sheet name="Form Fields" sheetId="5" r:id="rId9"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="50">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -918,6 +919,88 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{139F1479-2E59-4670-8557-FD1A600D9DD9}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.77734375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{172EB3BB-E440-4D9F-AB45-F40BA5013EFF}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -988,7 +1071,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54C0A2D9-C8FF-4F2E-9357-11D1A04AB716}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1059,7 +1142,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31F8298A-0165-44BF-9061-10BEE0A93A27}">
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Merged PR 2710: Merge Deepika_prod to master
</commit_message>
<xml_diff>
--- a/src/main/resources/Organizational_DeskReview_Field_Values.xlsx
+++ b/src/main/resources/Organizational_DeskReview_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21727"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C549426-EBDA-47CA-BD97-FB7828A38ECB}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53DA0360-8FF9-43CA-9C55-A0A6EE758A3D}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="6" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="5" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -18,9 +18,10 @@
     <sheet name="Award" sheetId="9" r:id="rId3"/>
     <sheet name="Sheet1" sheetId="4" r:id="rId4"/>
     <sheet name="Edition" sheetId="3" r:id="rId5"/>
-    <sheet name="Program" sheetId="6" r:id="rId6"/>
-    <sheet name="Fiscal" sheetId="7" r:id="rId7"/>
-    <sheet name="Form Fields" sheetId="5" r:id="rId8"/>
+    <sheet name="Edition1" sheetId="10" r:id="rId6"/>
+    <sheet name="Program" sheetId="6" r:id="rId7"/>
+    <sheet name="Fiscal" sheetId="7" r:id="rId8"/>
+    <sheet name="Form Fields" sheetId="5" r:id="rId9"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="50">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -918,6 +919,88 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{139F1479-2E59-4670-8557-FD1A600D9DD9}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.77734375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{172EB3BB-E440-4D9F-AB45-F40BA5013EFF}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -988,7 +1071,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54C0A2D9-C8FF-4F2E-9357-11D1A04AB716}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1059,7 +1142,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31F8298A-0165-44BF-9061-10BEE0A93A27}">
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
rafctored negotiation, closoeut, desk review, site review and sanity
</commit_message>
<xml_diff>
--- a/src/main/resources/Organizational_DeskReview_Field_Values.xlsx
+++ b/src/main/resources/Organizational_DeskReview_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Product\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA620691-8A42-4375-9F1E-FE8DB153FC52}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FC2315C-900F-403B-BCE8-27CE7168B71E}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12570" activeTab="6" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="53">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -186,6 +186,12 @@
   </si>
   <si>
     <t>Automation Runtime Desk Review Org level</t>
+  </si>
+  <si>
+    <t>Fiscal</t>
+  </si>
+  <si>
+    <t>Program</t>
   </si>
 </sst>
 </file>
@@ -545,13 +551,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27F20A35-8E6F-4015-873C-76781E4C62A4}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -562,7 +568,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -573,7 +579,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -584,7 +590,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -595,7 +601,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -614,15 +620,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F7BC2C8-C330-4CF5-B350-FDF7466963B4}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" style="1"/>
-    <col min="2" max="2" width="20.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="8.6640625" style="1"/>
+    <col min="1" max="1" width="8.7109375" style="1"/>
+    <col min="2" max="2" width="20.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -633,7 +639,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -644,7 +650,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -655,7 +661,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -666,7 +672,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -685,15 +691,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{661F5711-50C5-4AD1-966A-EEB6DD06A5CB}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" style="1"/>
-    <col min="2" max="2" width="20.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="8.6640625" style="1"/>
+    <col min="1" max="1" width="8.7109375" style="1"/>
+    <col min="2" max="2" width="20.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -704,7 +710,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -715,7 +721,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -726,7 +732,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -737,7 +743,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -756,12 +762,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFC7A54C-E16D-458B-92CE-DB4DE5E21708}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -769,7 +775,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -777,7 +783,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -785,7 +791,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -793,22 +799,22 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>27</v>
       </c>
@@ -821,14 +827,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4969FD67-2E2F-4920-8A24-9B3F6A7CB976}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -839,7 +845,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
@@ -850,7 +856,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
@@ -861,7 +867,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -872,7 +878,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -883,7 +889,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -894,7 +900,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -905,7 +911,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
@@ -924,15 +930,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{139F1479-2E59-4670-8557-FD1A600D9DD9}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="8.6640625" style="1"/>
+    <col min="1" max="1" width="8.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -943,7 +949,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
@@ -954,7 +960,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
@@ -965,7 +971,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -976,7 +982,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -987,7 +993,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -1006,15 +1012,15 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{172EB3BB-E440-4D9F-AB45-F40BA5013EFF}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" style="1"/>
-    <col min="2" max="2" width="20.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="8.6640625" style="1"/>
+    <col min="1" max="1" width="8.7109375" style="1"/>
+    <col min="2" max="2" width="20.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1025,7 +1031,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -1036,7 +1042,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1047,7 +1053,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -1055,10 +1061,10 @@
         <v>11</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -1077,15 +1083,15 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54C0A2D9-C8FF-4F2E-9357-11D1A04AB716}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" style="1"/>
-    <col min="2" max="2" width="20.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="8.6640625" style="1"/>
+    <col min="1" max="1" width="8.7109375" style="1"/>
+    <col min="2" max="2" width="20.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1096,7 +1102,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -1107,7 +1113,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1118,7 +1124,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -1126,10 +1132,10 @@
         <v>11</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -1148,14 +1154,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31F8298A-0165-44BF-9061-10BEE0A93A27}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.33203125" customWidth="1"/>
-    <col min="3" max="3" width="100.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.28515625" customWidth="1"/>
+    <col min="3" max="3" width="100.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1166,7 +1172,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1177,7 +1183,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1188,7 +1194,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -1199,7 +1205,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -1210,7 +1216,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -1221,7 +1227,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
@@ -1232,7 +1238,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
@@ -1243,7 +1249,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>4</v>
       </c>
@@ -1254,7 +1260,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>

</xml_diff>